<commit_message>
data: IDs dinámicos, campos detectados y reglas de validación actualizados (patente de Perú de 15 caracteres)
</commit_message>
<xml_diff>
--- a/data/Field_Validation_URLs.xlsx
+++ b/data/Field_Validation_URLs.xlsx
@@ -350,8 +350,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -374,7 +382,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -382,17 +390,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -692,13 +718,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -706,7 +732,7 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -714,7 +740,7 @@
       <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -722,7 +748,7 @@
       <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -730,7 +756,7 @@
       <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -738,7 +764,7 @@
       <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -746,7 +772,7 @@
       <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -754,7 +780,7 @@
       <c r="B8" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -762,7 +788,7 @@
       <c r="B9" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -770,7 +796,7 @@
       <c r="B10" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
     </row>
@@ -778,7 +804,7 @@
       <c r="B11" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -786,7 +812,7 @@
       <c r="B12" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -794,7 +820,7 @@
       <c r="B13" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -802,7 +828,7 @@
       <c r="B14" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -810,7 +836,7 @@
       <c r="B15" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -818,7 +844,7 @@
       <c r="B16" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -826,7 +852,7 @@
       <c r="B17" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -834,7 +860,7 @@
       <c r="B18" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -842,7 +868,7 @@
       <c r="B19" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -850,7 +876,7 @@
       <c r="B20" t="s">
         <v>4</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -858,7 +884,7 @@
       <c r="B21" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -866,7 +892,7 @@
       <c r="B22" t="s">
         <v>4</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -874,7 +900,7 @@
       <c r="B23" t="s">
         <v>4</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
         <v>31</v>
       </c>
     </row>
@@ -882,7 +908,7 @@
       <c r="B24" t="s">
         <v>4</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -890,7 +916,7 @@
       <c r="B25" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -898,7 +924,7 @@
       <c r="B26" t="s">
         <v>4</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>34</v>
       </c>
     </row>
@@ -906,7 +932,7 @@
       <c r="B27" t="s">
         <v>4</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -914,7 +940,7 @@
       <c r="B28" t="s">
         <v>4</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>36</v>
       </c>
     </row>
@@ -922,7 +948,7 @@
       <c r="B29" t="s">
         <v>4</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -930,7 +956,7 @@
       <c r="B30" t="s">
         <v>5</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="2" t="s">
         <v>38</v>
       </c>
     </row>
@@ -938,7 +964,7 @@
       <c r="B31" t="s">
         <v>5</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="2" t="s">
         <v>39</v>
       </c>
     </row>
@@ -946,7 +972,7 @@
       <c r="B32" t="s">
         <v>5</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -954,7 +980,7 @@
       <c r="B33" t="s">
         <v>5</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="2" t="s">
         <v>41</v>
       </c>
     </row>
@@ -962,7 +988,7 @@
       <c r="B34" t="s">
         <v>5</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="2" t="s">
         <v>42</v>
       </c>
     </row>
@@ -970,7 +996,7 @@
       <c r="B35" t="s">
         <v>5</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -978,7 +1004,7 @@
       <c r="B36" t="s">
         <v>5</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -986,7 +1012,7 @@
       <c r="B37" t="s">
         <v>5</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -994,7 +1020,7 @@
       <c r="B38" t="s">
         <v>5</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="2" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1002,7 +1028,7 @@
       <c r="B39" t="s">
         <v>5</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="2" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1010,7 +1036,7 @@
       <c r="B40" t="s">
         <v>5</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="2" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1018,7 +1044,7 @@
       <c r="B41" t="s">
         <v>5</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1026,7 +1052,7 @@
       <c r="B42" t="s">
         <v>5</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="2" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1034,7 +1060,7 @@
       <c r="B43" t="s">
         <v>6</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1042,7 +1068,7 @@
       <c r="B44" t="s">
         <v>6</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1050,7 +1076,7 @@
       <c r="B45" t="s">
         <v>6</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1058,7 +1084,7 @@
       <c r="B46" t="s">
         <v>6</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" s="2" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1066,7 +1092,7 @@
       <c r="B47" t="s">
         <v>6</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1074,7 +1100,7 @@
       <c r="B48" t="s">
         <v>6</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" s="2" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1082,7 +1108,7 @@
       <c r="B49" t="s">
         <v>6</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="2" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1090,7 +1116,7 @@
       <c r="B50" t="s">
         <v>6</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1098,7 +1124,7 @@
       <c r="B51" t="s">
         <v>6</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C51" s="2" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1106,7 +1132,7 @@
       <c r="B52" t="s">
         <v>6</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" s="2" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1114,7 +1140,7 @@
       <c r="B53" t="s">
         <v>6</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C53" s="2" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1122,7 +1148,7 @@
       <c r="B54" t="s">
         <v>7</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" s="2" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1130,7 +1156,7 @@
       <c r="B55" t="s">
         <v>7</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" s="2" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1138,7 +1164,7 @@
       <c r="B56" t="s">
         <v>7</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1146,7 +1172,7 @@
       <c r="B57" t="s">
         <v>7</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1154,7 +1180,7 @@
       <c r="B58" t="s">
         <v>7</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C58" s="2" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1162,7 +1188,7 @@
       <c r="B59" t="s">
         <v>7</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C59" s="2" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1170,7 +1196,7 @@
       <c r="B60" t="s">
         <v>7</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C60" s="2" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1178,7 +1204,7 @@
       <c r="B61" t="s">
         <v>7</v>
       </c>
-      <c r="C61" s="1" t="s">
+      <c r="C61" s="2" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1186,7 +1212,7 @@
       <c r="B62" t="s">
         <v>7</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="C62" s="2" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1194,7 +1220,7 @@
       <c r="B63" t="s">
         <v>7</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C63" s="2" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1202,7 +1228,7 @@
       <c r="B64" t="s">
         <v>7</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C64" s="2" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1210,7 +1236,7 @@
       <c r="B65" t="s">
         <v>7</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C65" s="2" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1218,7 +1244,7 @@
       <c r="B66" t="s">
         <v>7</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="C66" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1226,7 +1252,7 @@
       <c r="B67" t="s">
         <v>7</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C67" s="2" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1234,7 +1260,7 @@
       <c r="B68" t="s">
         <v>7</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C68" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1242,7 +1268,7 @@
       <c r="B69" t="s">
         <v>7</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C69" s="2" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1250,7 +1276,7 @@
       <c r="B70" t="s">
         <v>8</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="C70" s="2" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1258,7 +1284,7 @@
       <c r="B71" t="s">
         <v>8</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C71" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1266,7 +1292,7 @@
       <c r="B72" t="s">
         <v>8</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C72" s="2" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1274,7 +1300,7 @@
       <c r="B73" t="s">
         <v>8</v>
       </c>
-      <c r="C73" s="1" t="s">
+      <c r="C73" s="2" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1282,7 +1308,7 @@
       <c r="B74" t="s">
         <v>8</v>
       </c>
-      <c r="C74" s="1" t="s">
+      <c r="C74" s="2" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1290,7 +1316,7 @@
       <c r="B75" t="s">
         <v>8</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C75" s="2" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1298,7 +1324,7 @@
       <c r="B76" t="s">
         <v>8</v>
       </c>
-      <c r="C76" s="1" t="s">
+      <c r="C76" s="2" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1306,7 +1332,7 @@
       <c r="B77" t="s">
         <v>8</v>
       </c>
-      <c r="C77" s="1" t="s">
+      <c r="C77" s="2" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1314,7 +1340,7 @@
       <c r="B78" t="s">
         <v>8</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="C78" s="2" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1322,7 +1348,7 @@
       <c r="B79" t="s">
         <v>8</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C79" s="2" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1330,7 +1356,7 @@
       <c r="B80" t="s">
         <v>8</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C80" s="2" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1338,7 +1364,7 @@
       <c r="B81" t="s">
         <v>8</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="C81" s="2" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1346,7 +1372,7 @@
       <c r="B82" t="s">
         <v>8</v>
       </c>
-      <c r="C82" s="1" t="s">
+      <c r="C82" s="2" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1354,7 +1380,7 @@
       <c r="B83" t="s">
         <v>8</v>
       </c>
-      <c r="C83" s="1" t="s">
+      <c r="C83" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1362,7 +1388,7 @@
       <c r="B84" t="s">
         <v>8</v>
       </c>
-      <c r="C84" s="1" t="s">
+      <c r="C84" s="2" t="s">
         <v>91</v>
       </c>
     </row>
@@ -1370,7 +1396,7 @@
       <c r="B85" t="s">
         <v>9</v>
       </c>
-      <c r="C85" s="1" t="s">
+      <c r="C85" s="2" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1378,7 +1404,7 @@
       <c r="B86" t="s">
         <v>9</v>
       </c>
-      <c r="C86" s="1" t="s">
+      <c r="C86" s="2" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1386,7 +1412,7 @@
       <c r="B87" t="s">
         <v>9</v>
       </c>
-      <c r="C87" s="1" t="s">
+      <c r="C87" s="2" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1394,7 +1420,7 @@
       <c r="B88" t="s">
         <v>9</v>
       </c>
-      <c r="C88" s="1" t="s">
+      <c r="C88" s="2" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1402,7 +1428,7 @@
       <c r="B89" t="s">
         <v>9</v>
       </c>
-      <c r="C89" s="1" t="s">
+      <c r="C89" s="2" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1410,7 +1436,7 @@
       <c r="B90" t="s">
         <v>9</v>
       </c>
-      <c r="C90" s="1" t="s">
+      <c r="C90" s="2" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1418,7 +1444,7 @@
       <c r="B91" t="s">
         <v>9</v>
       </c>
-      <c r="C91" s="1" t="s">
+      <c r="C91" s="2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1426,7 +1452,7 @@
       <c r="B92" t="s">
         <v>9</v>
       </c>
-      <c r="C92" s="1" t="s">
+      <c r="C92" s="2" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1434,7 +1460,7 @@
       <c r="B93" t="s">
         <v>9</v>
       </c>
-      <c r="C93" s="1" t="s">
+      <c r="C93" s="2" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1442,7 +1468,7 @@
       <c r="B94" t="s">
         <v>9</v>
       </c>
-      <c r="C94" s="1" t="s">
+      <c r="C94" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1450,7 +1476,7 @@
       <c r="B95" t="s">
         <v>9</v>
       </c>
-      <c r="C95" s="1" t="s">
+      <c r="C95" s="2" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1458,7 +1484,7 @@
       <c r="B96" t="s">
         <v>10</v>
       </c>
-      <c r="C96" s="1" t="s">
+      <c r="C96" s="2" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1466,7 +1492,7 @@
       <c r="B97" t="s">
         <v>10</v>
       </c>
-      <c r="C97" s="1" t="s">
+      <c r="C97" s="2" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1474,7 +1500,7 @@
       <c r="B98" t="s">
         <v>10</v>
       </c>
-      <c r="C98" s="1" t="s">
+      <c r="C98" s="2" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1482,7 +1508,7 @@
       <c r="B99" t="s">
         <v>10</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="C99" s="2" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1490,7 +1516,7 @@
       <c r="B100" t="s">
         <v>10</v>
       </c>
-      <c r="C100" s="1" t="s">
+      <c r="C100" s="2" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1498,7 +1524,7 @@
       <c r="B101" t="s">
         <v>10</v>
       </c>
-      <c r="C101" s="1" t="s">
+      <c r="C101" s="2" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1506,7 +1532,7 @@
       <c r="B102" t="s">
         <v>10</v>
       </c>
-      <c r="C102" s="1" t="s">
+      <c r="C102" s="2" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>